<commit_message>
Add city/province and country autocomplete for vacation leave location
</commit_message>
<xml_diff>
--- a/backend/resources/templates/cs-form-6.xlsx
+++ b/backend/resources/templates/cs-form-6.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingia\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\ENHS-Leave-Management-System\backend\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7E8C38D-5ED0-4617-AE29-20CA3140F0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0E6ED1-9842-4998-904B-D2BFF2B91DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="CS Form No. 6, Rev 2020 2 of 2" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'CS Form No. 6, Rev 2020 1 of 2'!$A$1:$I$65</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'CS Form No. 6, Rev 2020 1 of 2'!$A$1:$I$66</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'CS Form No. 6, Rev 2020 2 of 2'!$A$1:$K$62</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
@@ -390,9 +390,6 @@
     <t>Abroad (Specify) _____________________________</t>
   </si>
   <si>
-    <t>School Principal I</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">
 _________________________________
@@ -465,6 +462,9 @@
   </si>
   <si>
     <t>2.  NAME :                    (Last)                                   (First)                         (Middle)</t>
+  </si>
+  <si>
+    <t>School Principal II</t>
   </si>
 </sst>
 </file>
@@ -899,7 +899,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -938,9 +938,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1000,6 +997,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1047,18 +1065,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3250,13 +3256,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1950363</xdr:colOff>
+      <xdr:colOff>1804572</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>95230</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>2649466</xdr:colOff>
+      <xdr:colOff>2503675</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>293667</xdr:rowOff>
     </xdr:to>
@@ -3273,7 +3279,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6408063" y="2257405"/>
+          <a:off x="6275490" y="2252934"/>
           <a:ext cx="699103" cy="198437"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4347,16 +4353,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>7937</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>75974</xdr:colOff>
       <xdr:row>58</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>217714</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>3000374</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>357188</xdr:rowOff>
+      <xdr:colOff>2898321</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>10206</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4371,15 +4377,13 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4468812" y="9977438"/>
+          <a:off x="4355420" y="10048875"/>
           <a:ext cx="2992437" cy="214313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
+        <a:noFill/>
         <a:ln w="9525" cmpd="sng">
           <a:noFill/>
         </a:ln>
@@ -4403,7 +4407,24 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>EMILY O.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t> BENITEZ</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -4915,6 +4936,153 @@
         <a:lstStyle/>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>316819</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>240846</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>948417</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>33338</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609373" y="10072007"/>
+          <a:ext cx="2992437" cy="214313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>PRECIOUS</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t> C. PABON</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>772660</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>615042</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>805543</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>829355</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2262642" y="11908971"/>
+          <a:ext cx="2992437" cy="214313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>RACHELE R. LLANA, PhD, CESO V</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -5268,47 +5436,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="63" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="50"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="49"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="55" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="N2" s="44"/>
+      <c r="A2" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="N2" s="43"/>
     </row>
     <row r="3" spans="1:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
       <c r="J3" s="1"/>
-      <c r="N3" s="44"/>
+      <c r="N3" s="43"/>
     </row>
     <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
@@ -5318,7 +5486,7 @@
       <c r="C4" s="4"/>
       <c r="D4" s="23"/>
       <c r="E4" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -5330,14 +5498,14 @@
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="65"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66"/>
-      <c r="I5" s="67"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="72"/>
+      <c r="I5" s="73"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -5347,7 +5515,7 @@
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="34" t="s">
         <v>29</v>
       </c>
       <c r="G6" s="4"/>
@@ -5367,19 +5535,19 @@
       <c r="I7" s="9"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:14" s="38" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="36"/>
-      <c r="B8" s="62" t="s">
+    <row r="8" spans="1:14" s="37" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35"/>
+      <c r="B8" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="63"/>
-      <c r="J8" s="37"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="68"/>
+      <c r="I8" s="69"/>
+      <c r="J8" s="36"/>
     </row>
     <row r="9" spans="1:14" ht="19.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
@@ -5390,7 +5558,7 @@
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
       <c r="F9" s="14"/>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="48" t="s">
         <v>18</v>
       </c>
       <c r="H9" s="13"/>
@@ -5412,12 +5580,12 @@
     <row r="11" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="47" t="s">
+      <c r="C11" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="48"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="47"/>
       <c r="G11" s="2"/>
       <c r="H11" s="29" t="s">
         <v>31</v>
@@ -5429,10 +5597,10 @@
     <row r="12" spans="1:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="2"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="48"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="47"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="9"/>
@@ -5441,15 +5609,15 @@
     <row r="13" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="8"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="47" t="s">
+      <c r="C13" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="47"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="48"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="47"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="48" t="s">
+      <c r="I13" s="47" t="s">
         <v>14</v>
       </c>
       <c r="J13" s="1"/>
@@ -5458,27 +5626,27 @@
     <row r="14" spans="1:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
       <c r="B14" s="2"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="48"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="47"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="48"/>
+      <c r="I14" s="47"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="47" t="s">
+      <c r="C15" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="47"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="48"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="47"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="48" t="s">
+      <c r="I15" s="47" t="s">
         <v>64</v>
       </c>
       <c r="J15" s="1"/>
@@ -5486,10 +5654,10 @@
     <row r="16" spans="1:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="48"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="47"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="9"/>
@@ -5498,26 +5666,26 @@
     <row r="17" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="47" t="s">
+      <c r="C17" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="47"/>
-      <c r="E17" s="47"/>
-      <c r="F17" s="48"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="47"/>
       <c r="G17" s="2"/>
       <c r="H17" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="31"/>
+      <c r="I17" s="30"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="47"/>
-      <c r="F18" s="48"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="47"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="9"/>
@@ -5525,15 +5693,15 @@
     </row>
     <row r="19" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
-      <c r="C19" s="47" t="s">
+      <c r="C19" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="48"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="47"/>
       <c r="G19" s="2"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="48" t="s">
+      <c r="H19" s="50"/>
+      <c r="I19" s="47" t="s">
         <v>57</v>
       </c>
       <c r="J19" s="1"/>
@@ -5541,26 +5709,26 @@
     <row r="20" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="48"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="47"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-      <c r="I20" s="48"/>
+      <c r="I20" s="47"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
-      <c r="C21" s="47" t="s">
+      <c r="C21" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="48"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="47"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="48" t="s">
+      <c r="I21" s="47" t="s">
         <v>63</v>
       </c>
       <c r="J21" s="1"/>
@@ -5570,10 +5738,10 @@
     <row r="22" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="48"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="47"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="9"/>
@@ -5585,12 +5753,12 @@
     <row r="23" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="47" t="s">
+      <c r="C23" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="48"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="47"/>
       <c r="H23" s="2" t="s">
         <v>24</v>
       </c>
@@ -5600,10 +5768,10 @@
     <row r="24" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="8"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="48"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="47"/>
       <c r="G24" s="2"/>
       <c r="I24" s="27"/>
       <c r="J24" s="1"/>
@@ -5613,12 +5781,12 @@
     <row r="25" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="47" t="s">
+      <c r="C25" s="46" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="48"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="47"/>
       <c r="G25" s="2"/>
       <c r="H25" s="29" t="s">
         <v>22</v>
@@ -5631,10 +5799,10 @@
     <row r="26" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="8"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="48"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="47"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="27"/>
@@ -5646,12 +5814,12 @@
     <row r="27" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="8"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="47" t="s">
+      <c r="C27" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="48"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="47"/>
       <c r="G27" s="2"/>
       <c r="H27" s="9" t="s">
         <v>58</v>
@@ -5664,10 +5832,10 @@
     <row r="28" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="8"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="48"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="47"/>
       <c r="G28" s="2"/>
       <c r="I28" s="27"/>
       <c r="J28" s="1"/>
@@ -5678,12 +5846,12 @@
     <row r="29" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="8"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="47" t="s">
+      <c r="C29" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="48"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="47"/>
       <c r="G29" s="2"/>
       <c r="H29" t="s">
         <v>24</v>
@@ -5694,10 +5862,10 @@
     <row r="30" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="8"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="48"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="47"/>
       <c r="G30" s="2"/>
       <c r="I30" s="27"/>
       <c r="J30" s="1"/>
@@ -5707,12 +5875,12 @@
     <row r="31" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="53" t="s">
+      <c r="C31" s="59" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="60"/>
       <c r="G31" s="2"/>
       <c r="H31" s="29" t="s">
         <v>20</v>
@@ -5725,10 +5893,10 @@
     <row r="32" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="8"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="48"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="47"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="9"/>
@@ -5740,15 +5908,15 @@
     <row r="33" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="8"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="47" t="s">
+      <c r="C33" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="47"/>
-      <c r="E33" s="47"/>
-      <c r="F33" s="48"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="47"/>
       <c r="G33" s="2"/>
-      <c r="H33" s="51"/>
-      <c r="I33" s="48" t="s">
+      <c r="H33" s="50"/>
+      <c r="I33" s="47" t="s">
         <v>32</v>
       </c>
       <c r="J33" s="1"/>
@@ -5764,13 +5932,13 @@
       <c r="F34" s="9"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-      <c r="I34" s="48"/>
+      <c r="I34" s="47"/>
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="47" t="s">
+      <c r="C35" s="46" t="s">
         <v>56</v>
       </c>
       <c r="D35" s="2"/>
@@ -5778,7 +5946,7 @@
       <c r="F35" s="9"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="48" t="s">
+      <c r="I35" s="47" t="s">
         <v>21</v>
       </c>
       <c r="J35" s="1"/>
@@ -5786,7 +5954,7 @@
     <row r="36" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="47"/>
+      <c r="C36" s="46"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="9"/>
@@ -5797,7 +5965,7 @@
     <row r="37" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="8"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="47"/>
+      <c r="C37" s="46"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="9"/>
@@ -5831,7 +5999,7 @@
       <c r="F39" s="9"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
-      <c r="I39" s="48" t="s">
+      <c r="I39" s="47" t="s">
         <v>16</v>
       </c>
       <c r="J39" s="1"/>
@@ -5845,7 +6013,7 @@
       <c r="F40" s="9"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
-      <c r="I40" s="48"/>
+      <c r="I40" s="47"/>
       <c r="J40" s="1"/>
     </row>
     <row r="41" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -5859,7 +6027,7 @@
       <c r="F41" s="9"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
-      <c r="I41" s="48" t="s">
+      <c r="I41" s="47" t="s">
         <v>30</v>
       </c>
       <c r="J41" s="1"/>
@@ -5904,7 +6072,7 @@
     </row>
     <row r="45" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="8"/>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="31" t="s">
         <v>25</v>
       </c>
       <c r="C45" s="2"/>
@@ -5913,7 +6081,7 @@
       <c r="F45" s="9"/>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
-      <c r="I45" s="48" t="s">
+      <c r="I45" s="47" t="s">
         <v>2</v>
       </c>
       <c r="J45" s="1"/>
@@ -5927,12 +6095,12 @@
       <c r="F46" s="9"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
-      <c r="I46" s="48"/>
+      <c r="I46" s="47"/>
       <c r="J46" s="1"/>
     </row>
     <row r="47" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="8"/>
-      <c r="B47" s="32"/>
+      <c r="B47" s="31"/>
       <c r="C47" s="2" t="s">
         <v>17</v>
       </c>
@@ -5941,19 +6109,19 @@
       <c r="F47" s="9"/>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
-      <c r="I47" s="48" t="s">
+      <c r="I47" s="47" t="s">
         <v>3</v>
       </c>
       <c r="J47" s="1"/>
     </row>
     <row r="48" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="8"/>
-      <c r="B48" s="34" t="s">
+      <c r="B48" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="C48" s="33"/>
-      <c r="D48" s="33"/>
-      <c r="E48" s="33"/>
+      <c r="C48" s="32"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="32"/>
       <c r="F48" s="9"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
@@ -5967,26 +6135,26 @@
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="9"/>
-      <c r="G49" s="64" t="s">
+      <c r="G49" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="H49" s="60"/>
-      <c r="I49" s="61"/>
+      <c r="H49" s="66"/>
+      <c r="I49" s="67"/>
       <c r="J49" s="1"/>
     </row>
-    <row r="50" spans="1:10" s="38" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="36"/>
-      <c r="B50" s="62" t="s">
+    <row r="50" spans="1:10" s="37" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="35"/>
+      <c r="B50" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="62"/>
-      <c r="D50" s="62"/>
-      <c r="E50" s="62"/>
-      <c r="F50" s="62"/>
-      <c r="G50" s="62"/>
-      <c r="H50" s="62"/>
-      <c r="I50" s="63"/>
-      <c r="J50" s="37"/>
+      <c r="C50" s="68"/>
+      <c r="D50" s="68"/>
+      <c r="E50" s="68"/>
+      <c r="F50" s="68"/>
+      <c r="G50" s="68"/>
+      <c r="H50" s="68"/>
+      <c r="I50" s="69"/>
+      <c r="J50" s="36"/>
     </row>
     <row r="51" spans="1:10" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
@@ -6018,7 +6186,7 @@
     </row>
     <row r="53" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="8"/>
-      <c r="C53" s="45" t="s">
+      <c r="C53" s="44" t="s">
         <v>40</v>
       </c>
       <c r="D53" s="2"/>
@@ -6064,7 +6232,7 @@
     <row r="56" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="8"/>
       <c r="B56" s="2"/>
-      <c r="C56" s="46" t="s">
+      <c r="C56" s="45" t="s">
         <v>36</v>
       </c>
       <c r="D56" s="17"/>
@@ -6080,7 +6248,7 @@
     <row r="57" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="8"/>
       <c r="B57" s="2"/>
-      <c r="C57" s="46" t="s">
+      <c r="C57" s="45" t="s">
         <v>37</v>
       </c>
       <c r="D57" s="17"/>
@@ -6096,7 +6264,7 @@
     <row r="58" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="8"/>
       <c r="B58" s="2"/>
-      <c r="C58" s="46" t="s">
+      <c r="C58" s="45" t="s">
         <v>38</v>
       </c>
       <c r="D58" s="17"/>
@@ -6123,21 +6291,21 @@
       </c>
       <c r="J59" s="1"/>
     </row>
-    <row r="60" spans="1:10" s="43" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="39"/>
-      <c r="B60" s="40"/>
-      <c r="C60" s="58" t="s">
+    <row r="60" spans="1:10" s="42" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="38"/>
+      <c r="B60" s="39"/>
+      <c r="C60" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="D60" s="58"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="41"/>
-      <c r="G60" s="59" t="s">
-        <v>65</v>
-      </c>
-      <c r="H60" s="60"/>
-      <c r="I60" s="61"/>
-      <c r="J60" s="42"/>
+      <c r="D60" s="64"/>
+      <c r="E60" s="64"/>
+      <c r="F60" s="40"/>
+      <c r="G60" s="65" t="s">
+        <v>68</v>
+      </c>
+      <c r="H60" s="66"/>
+      <c r="I60" s="67"/>
+      <c r="J60" s="41"/>
     </row>
     <row r="61" spans="1:10" ht="19.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
@@ -6201,92 +6369,86 @@
       <c r="J64" s="1"/>
     </row>
     <row r="65" spans="1:9" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="68" t="s">
-        <v>66</v>
-      </c>
-      <c r="B65" s="69"/>
-      <c r="C65" s="69"/>
-      <c r="D65" s="69"/>
-      <c r="E65" s="69"/>
-      <c r="F65" s="69"/>
-      <c r="G65" s="69"/>
-      <c r="H65" s="69"/>
-      <c r="I65" s="70"/>
+      <c r="A65" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="B65" s="55"/>
+      <c r="C65" s="55"/>
+      <c r="D65" s="55"/>
+      <c r="E65" s="55"/>
+      <c r="F65" s="55"/>
+      <c r="G65" s="55"/>
+      <c r="H65" s="55"/>
+      <c r="I65" s="56"/>
     </row>
     <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="A66" s="30"/>
-      <c r="B66" s="30"/>
-      <c r="C66" s="30"/>
-      <c r="D66" s="30"/>
-      <c r="E66" s="30"/>
-      <c r="F66" s="30"/>
-      <c r="G66" s="30"/>
-      <c r="H66" s="30"/>
-      <c r="I66" s="30"/>
+      <c r="A66" s="52"/>
+      <c r="B66" s="51"/>
+      <c r="C66" s="51"/>
+      <c r="D66" s="51"/>
+      <c r="E66" s="51"/>
+      <c r="F66" s="51"/>
+      <c r="G66" s="51"/>
+      <c r="H66" s="51"/>
+      <c r="I66" s="53"/>
     </row>
     <row r="67" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="71"/>
-      <c r="B67" s="71"/>
-      <c r="C67" s="71"/>
-      <c r="D67" s="71"/>
-      <c r="E67" s="71"/>
-      <c r="F67" s="71"/>
-      <c r="G67" s="71"/>
-      <c r="H67" s="71"/>
-      <c r="I67" s="71"/>
+      <c r="A67" s="57"/>
+      <c r="B67" s="57"/>
+      <c r="C67" s="57"/>
+      <c r="D67" s="57"/>
+      <c r="E67" s="57"/>
+      <c r="F67" s="57"/>
+      <c r="G67" s="57"/>
+      <c r="H67" s="57"/>
+      <c r="I67" s="57"/>
     </row>
     <row r="68" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="71"/>
-      <c r="B68" s="71"/>
-      <c r="C68" s="71"/>
-      <c r="D68" s="71"/>
-      <c r="E68" s="71"/>
-      <c r="F68" s="71"/>
-      <c r="G68" s="71"/>
-      <c r="H68" s="71"/>
-      <c r="I68" s="71"/>
+      <c r="A68" s="57"/>
+      <c r="B68" s="57"/>
+      <c r="C68" s="57"/>
+      <c r="D68" s="57"/>
+      <c r="E68" s="57"/>
+      <c r="F68" s="57"/>
+      <c r="G68" s="57"/>
+      <c r="H68" s="57"/>
+      <c r="I68" s="57"/>
     </row>
     <row r="69" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="71"/>
-      <c r="B69" s="71"/>
-      <c r="C69" s="71"/>
-      <c r="D69" s="71"/>
-      <c r="E69" s="71"/>
-      <c r="F69" s="71"/>
-      <c r="G69" s="71"/>
-      <c r="H69" s="71"/>
-      <c r="I69" s="71"/>
+      <c r="A69" s="57"/>
+      <c r="B69" s="57"/>
+      <c r="C69" s="57"/>
+      <c r="D69" s="57"/>
+      <c r="E69" s="57"/>
+      <c r="F69" s="57"/>
+      <c r="G69" s="57"/>
+      <c r="H69" s="57"/>
+      <c r="I69" s="57"/>
     </row>
     <row r="70" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="71"/>
-      <c r="B70" s="71"/>
-      <c r="C70" s="71"/>
-      <c r="D70" s="71"/>
-      <c r="E70" s="71"/>
-      <c r="F70" s="71"/>
-      <c r="G70" s="71"/>
-      <c r="H70" s="71"/>
-      <c r="I70" s="71"/>
+      <c r="A70" s="57"/>
+      <c r="B70" s="57"/>
+      <c r="C70" s="57"/>
+      <c r="D70" s="57"/>
+      <c r="E70" s="57"/>
+      <c r="F70" s="57"/>
+      <c r="G70" s="57"/>
+      <c r="H70" s="57"/>
+      <c r="I70" s="57"/>
     </row>
     <row r="71" spans="1:9" s="28" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="71"/>
-      <c r="B71" s="71"/>
-      <c r="C71" s="71"/>
-      <c r="D71" s="71"/>
-      <c r="E71" s="71"/>
-      <c r="F71" s="71"/>
-      <c r="G71" s="71"/>
-      <c r="H71" s="71"/>
-      <c r="I71" s="71"/>
+      <c r="A71" s="57"/>
+      <c r="B71" s="57"/>
+      <c r="C71" s="57"/>
+      <c r="D71" s="57"/>
+      <c r="E71" s="57"/>
+      <c r="F71" s="57"/>
+      <c r="G71" s="57"/>
+      <c r="H71" s="57"/>
+      <c r="I71" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A65:I65"/>
-    <mergeCell ref="A67:I67"/>
-    <mergeCell ref="A68:I68"/>
-    <mergeCell ref="A69:I69"/>
-    <mergeCell ref="A71:I71"/>
-    <mergeCell ref="A70:I70"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="A2:I2"/>
@@ -6298,6 +6460,12 @@
     <mergeCell ref="B50:I50"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A65:I65"/>
+    <mergeCell ref="A67:I67"/>
+    <mergeCell ref="A68:I68"/>
+    <mergeCell ref="A69:I69"/>
+    <mergeCell ref="A71:I71"/>
+    <mergeCell ref="A70:I70"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.5" right="0.5" top="0.25" bottom="0" header="0.5" footer="0.5"/>

</xml_diff>